<commit_message>
Update attendance sheet for Engenharia de Software 2026-27
</commit_message>
<xml_diff>
--- a/Folha_de_Presencas_Engenharia_de_Software_2026-27.xlsx
+++ b/Folha_de_Presencas_Engenharia_de_Software_2026-27.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18600" windowHeight="6800"/>
+    <workbookView windowWidth="19200" windowHeight="6800"/>
   </bookViews>
   <sheets>
     <sheet name="Presenças" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="32">
   <si>
     <t>REGISTO DE PRESENÇAS</t>
   </si>
@@ -101,7 +101,7 @@
     <t>Marina Archeli Perez</t>
   </si>
   <si>
-    <t>Thaniel Pedro</t>
+    <t>Thaniel Jorge Guimarães Pedro</t>
   </si>
   <si>
     <t>13422</t>
@@ -116,7 +116,7 @@
     <t>Registos por aula</t>
   </si>
   <si>
-    <t>X  Presente     F  Falta     J  Falta justificada     ·     Célula vazia: ainda por registar</t>
+    <t>P  Presente     F  Falta     J  Falta justificada     ·     Célula vazia: ainda por registar</t>
   </si>
   <si>
     <t>24/12 e 31/12 coincidem com as férias de Natal. Essas datas foram excluídas.</t>
@@ -360,7 +360,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -399,12 +399,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFE7EFF1"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -596,7 +590,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="39">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -780,6 +774,19 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD5E0E4"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDCE5E9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDCE5E9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFD5E0E4"/>
       </left>
@@ -860,6 +867,19 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD5E0E4"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDCE5E9"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFD5E0E4"/>
       </left>
@@ -931,6 +951,19 @@
         <color rgb="FFE8E5DB"/>
       </left>
       <right/>
+      <top style="thin">
+        <color rgb="FFDCE5E9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB8C8CF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD5E0E4"/>
+      </right>
       <top style="thin">
         <color rgb="FFDCE5E9"/>
       </top>
@@ -1100,7 +1133,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="31" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="34" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1112,119 +1145,119 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="32" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="32" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="33" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="35" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="35" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="36" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="34" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="35" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="34" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="36" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="37" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="37" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="38" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="37" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="39" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="40" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1313,20 +1346,20 @@
     <xf numFmtId="0" fontId="8" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1334,37 +1367,46 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2115,7 +2157,9 @@
         <v>17</v>
       </c>
       <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
+      <c r="E8" s="18" t="s">
+        <v>17</v>
+      </c>
       <c r="F8" s="18"/>
       <c r="G8" s="18"/>
       <c r="H8" s="18"/>
@@ -2129,8 +2173,8 @@
       <c r="P8" s="18"/>
       <c r="Q8" s="19"/>
       <c r="R8" s="20">
-        <f t="shared" ref="R8:R13" si="0">COUNTIF(C8:Q8,"X")</f>
-        <v>1</v>
+        <f>COUNTIF(C8:Q8,"P")</f>
+        <v>0</v>
       </c>
       <c r="S8" s="21">
         <f>COUNTIF(C8:Q8,"F")</f>
@@ -2154,7 +2198,9 @@
       <c r="D9" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="26"/>
+      <c r="E9" s="26" t="s">
+        <v>17</v>
+      </c>
       <c r="F9" s="26"/>
       <c r="G9" s="26"/>
       <c r="H9" s="26"/>
@@ -2167,31 +2213,33 @@
       <c r="O9" s="26"/>
       <c r="P9" s="26"/>
       <c r="Q9" s="27"/>
-      <c r="R9" s="20">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="S9" s="28">
+      <c r="R9" s="28">
+        <f>COUNTIF(C9:Q9,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="S9" s="29">
         <f>COUNTIF(C9:Q9,"F")</f>
         <v>0</v>
       </c>
-      <c r="T9" s="29">
+      <c r="T9" s="30">
         <f>COUNTIF(C9:Q9,"J")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:20">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="32" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="17" t="s">
         <v>17</v>
       </c>
       <c r="D10" s="26"/>
-      <c r="E10" s="26"/>
+      <c r="E10" s="26" t="s">
+        <v>17</v>
+      </c>
       <c r="F10" s="26"/>
       <c r="G10" s="26"/>
       <c r="H10" s="26"/>
@@ -2204,15 +2252,15 @@
       <c r="O10" s="26"/>
       <c r="P10" s="26"/>
       <c r="Q10" s="27"/>
-      <c r="R10" s="20">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="S10" s="28">
+      <c r="R10" s="28">
+        <f>COUNTIF(C10:Q10,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="S10" s="29">
         <f>COUNTIF(C10:Q10,"F")</f>
         <v>0</v>
       </c>
-      <c r="T10" s="29">
+      <c r="T10" s="30">
         <f>COUNTIF(C10:Q10,"J")</f>
         <v>0</v>
       </c>
@@ -2241,85 +2289,88 @@
       <c r="O11" s="26"/>
       <c r="P11" s="26"/>
       <c r="Q11" s="27"/>
-      <c r="R11" s="20">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="S11" s="28">
+      <c r="R11" s="28">
+        <f>COUNTIF(C11:Q11,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="S11" s="29">
         <f>COUNTIF(C11:Q11,"F")</f>
         <v>0</v>
       </c>
-      <c r="T11" s="29">
+      <c r="T11" s="30">
         <f>COUNTIF(C11:Q11,"J")</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1" spans="1:20">
-      <c r="A12" s="32"/>
-      <c r="B12" s="33" t="s">
+      <c r="A12" s="33">
+        <v>13658</v>
+      </c>
+      <c r="B12" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="34" t="s">
+      <c r="C12" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="35" t="s">
+      <c r="D12" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-      <c r="K12" s="35"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="35"/>
-      <c r="N12" s="35"/>
-      <c r="O12" s="35"/>
-      <c r="P12" s="35"/>
-      <c r="Q12" s="36"/>
-      <c r="R12" s="20">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="S12" s="37"/>
-      <c r="T12" s="38"/>
+      <c r="E12" s="36" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="36"/>
+      <c r="L12" s="36"/>
+      <c r="M12" s="36"/>
+      <c r="N12" s="36"/>
+      <c r="O12" s="36"/>
+      <c r="P12" s="36"/>
+      <c r="Q12" s="37"/>
+      <c r="R12" s="38"/>
+      <c r="S12" s="39"/>
+      <c r="T12" s="40"/>
     </row>
     <row r="13" ht="34" customHeight="1" spans="1:20">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="40" t="s">
+      <c r="B13" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="41" t="s">
+      <c r="C13" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="42" t="s">
+      <c r="D13" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="42"/>
-      <c r="G13" s="42"/>
-      <c r="H13" s="42"/>
-      <c r="I13" s="42"/>
-      <c r="J13" s="42"/>
-      <c r="K13" s="42"/>
-      <c r="L13" s="42"/>
-      <c r="M13" s="42"/>
-      <c r="N13" s="42"/>
-      <c r="O13" s="42"/>
-      <c r="P13" s="42"/>
-      <c r="Q13" s="43"/>
-      <c r="R13" s="20">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="S13" s="44">
+      <c r="E13" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="44"/>
+      <c r="G13" s="44"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
+      <c r="N13" s="44"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="44"/>
+      <c r="Q13" s="45"/>
+      <c r="R13" s="46">
+        <f>COUNTIF(C13:Q13,"P")</f>
+        <v>0</v>
+      </c>
+      <c r="S13" s="47">
         <f>COUNTIF(C13:Q13,"F")</f>
         <v>0</v>
       </c>
-      <c r="T13" s="45">
+      <c r="T13" s="48">
         <f>COUNTIF(C13:Q13,"J")</f>
         <v>0</v>
       </c>
@@ -2347,79 +2398,79 @@
       <c r="T14" s="1"/>
     </row>
     <row r="15" ht="25" customHeight="1" spans="1:20">
-      <c r="A15" s="46"/>
-      <c r="B15" s="46" t="s">
+      <c r="A15" s="49"/>
+      <c r="B15" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="47">
+      <c r="C15" s="50">
         <f>COUNTIF(C8:C13,"X")+COUNTIF(C8:C13,"F")+COUNTIF(C8:C13,"J")</f>
         <v>6</v>
       </c>
-      <c r="D15" s="47">
+      <c r="D15" s="50">
         <f>COUNTIF(D8:D13,"X")+COUNTIF(D8:D13,"F")+COUNTIF(D8:D13,"J")</f>
         <v>3</v>
       </c>
-      <c r="E15" s="47">
-        <f t="shared" ref="E15:Q15" si="1">COUNTIF(E8:E13,"X")+COUNTIF(E8:E13,"F")+COUNTIF(E8:E13,"J")</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="G15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="H15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="L15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="M15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="N15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="O15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="47">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R15" s="47">
+      <c r="E15" s="50">
+        <f t="shared" ref="E15:Q15" si="0">COUNTIF(E8:E13,"X")+COUNTIF(E8:E13,"F")+COUNTIF(E8:E13,"J")</f>
+        <v>5</v>
+      </c>
+      <c r="F15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="50">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R15" s="50">
         <f>SUM(R8:R13)</f>
-        <v>9</v>
-      </c>
-      <c r="S15" s="47">
+        <v>0</v>
+      </c>
+      <c r="S15" s="50">
         <f>SUM(S8:S13)</f>
         <v>0</v>
       </c>
-      <c r="T15" s="47">
+      <c r="T15" s="50">
         <f>SUM(T8:T13)</f>
         <v>0</v>
       </c>
@@ -2447,7 +2498,7 @@
       <c r="T16" s="1"/>
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:20">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="51" t="s">
         <v>29</v>
       </c>
       <c r="B17" s="1"/>
@@ -2471,7 +2522,7 @@
       <c r="T17" s="1"/>
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:20">
-      <c r="A18" s="49" t="s">
+      <c r="A18" s="52" t="s">
         <v>30</v>
       </c>
       <c r="B18" s="1"/>
@@ -2495,7 +2546,7 @@
       <c r="T18" s="1"/>
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:20">
-      <c r="A19" s="50" t="s">
+      <c r="A19" s="53" t="s">
         <v>31</v>
       </c>
       <c r="B19" s="1"/>

</xml_diff>